<commit_message>
data: price.xlsx 현재가 업데이트 (2026-07-16 기준, 349/350 종목)
</commit_message>
<xml_diff>
--- a/data/price.xlsx
+++ b/data/price.xlsx
@@ -79988,1054 +79988,1054 @@
         <v>46234</v>
       </c>
       <c r="B80" t="n">
-        <v>285000</v>
+        <v>255000</v>
       </c>
       <c r="C80" t="n">
-        <v>2180000</v>
+        <v>1842000</v>
       </c>
       <c r="D80" t="n">
-        <v>1409000</v>
+        <v>1212000</v>
       </c>
       <c r="E80" t="n">
-        <v>194300</v>
+        <v>172000</v>
       </c>
       <c r="F80" t="n">
-        <v>1584000</v>
+        <v>1277000</v>
       </c>
       <c r="G80" t="n">
-        <v>457500</v>
+        <v>425000</v>
       </c>
       <c r="H80" t="n">
-        <v>326000</v>
+        <v>334000</v>
       </c>
       <c r="I80" t="n">
-        <v>340500</v>
+        <v>331000</v>
       </c>
       <c r="J80" t="n">
-        <v>184400</v>
+        <v>181100</v>
       </c>
       <c r="K80" t="n">
-        <v>1395000</v>
+        <v>1396000</v>
       </c>
       <c r="L80" t="n">
-        <v>391500</v>
+        <v>346000</v>
       </c>
       <c r="M80" t="n">
-        <v>147500</v>
+        <v>149700</v>
       </c>
       <c r="N80" t="n">
-        <v>504000</v>
+        <v>484000</v>
       </c>
       <c r="O80" t="n">
-        <v>109200</v>
+        <v>107900</v>
       </c>
       <c r="P80" t="n">
-        <v>78100</v>
+        <v>69700</v>
       </c>
       <c r="Q80" t="n">
-        <v>967000</v>
+        <v>943000</v>
       </c>
       <c r="R80" t="n">
-        <v>657000</v>
+        <v>580000</v>
       </c>
       <c r="S80" t="n">
-        <v>488000</v>
+        <v>482000</v>
       </c>
       <c r="T80" t="n">
-        <v>175200</v>
+        <v>175800</v>
       </c>
       <c r="U80" t="n">
-        <v>128500</v>
+        <v>136800</v>
       </c>
       <c r="V80" t="n">
-        <v>434000</v>
+        <v>434500</v>
       </c>
       <c r="W80" t="n">
-        <v>851000</v>
+        <v>797000</v>
       </c>
       <c r="X80" t="n">
-        <v>202500</v>
+        <v>190000</v>
       </c>
       <c r="Y80" t="n">
-        <v>191300</v>
+        <v>190000</v>
       </c>
       <c r="Z80" t="n">
-        <v>182400</v>
+        <v>179000</v>
       </c>
       <c r="AA80" t="n">
-        <v>648000</v>
+        <v>701000</v>
       </c>
       <c r="AB80" t="n">
-        <v>2924000</v>
+        <v>2789000</v>
       </c>
       <c r="AC80" t="n">
-        <v>81300</v>
+        <v>86700</v>
       </c>
       <c r="AD80" t="n">
-        <v>313500</v>
+        <v>311500</v>
       </c>
       <c r="AE80" t="n">
-        <v>340500</v>
+        <v>354000</v>
       </c>
       <c r="AF80" t="n">
-        <v>42200</v>
+        <v>40050</v>
       </c>
       <c r="AG80" t="n">
-        <v>36200</v>
+        <v>34050</v>
       </c>
       <c r="AH80" t="n">
-        <v>31450</v>
+        <v>31500</v>
       </c>
       <c r="AI80" t="n">
-        <v>1382000</v>
+        <v>1202000</v>
       </c>
       <c r="AJ80" t="n">
-        <v>1043000</v>
+        <v>1029000</v>
       </c>
       <c r="AK80" t="n">
-        <v>222000</v>
+        <v>242500</v>
       </c>
       <c r="AL80" t="n">
-        <v>22350</v>
+        <v>22300</v>
       </c>
       <c r="AM80" t="n">
-        <v>178900</v>
+        <v>159000</v>
       </c>
       <c r="AN80" t="n">
-        <v>115000</v>
+        <v>118300</v>
       </c>
       <c r="AO80" t="n">
-        <v>88700</v>
+        <v>89700</v>
       </c>
       <c r="AP80" t="n">
-        <v>264000</v>
+        <v>260500</v>
       </c>
       <c r="AQ80" t="n">
-        <v>19740</v>
+        <v>20050</v>
       </c>
       <c r="AR80" t="n">
-        <v>173500</v>
+        <v>179900</v>
       </c>
       <c r="AS80" t="n">
-        <v>742000</v>
+        <v>668000</v>
       </c>
       <c r="AT80" t="n">
-        <v>102900</v>
+        <v>121400</v>
       </c>
       <c r="AU80" t="n">
-        <v>21250</v>
+        <v>21600</v>
       </c>
       <c r="AV80" t="n">
         <v>749000</v>
       </c>
       <c r="AW80" t="n">
-        <v>199500</v>
+        <v>204500</v>
       </c>
       <c r="AX80" t="n">
-        <v>35350</v>
+        <v>35900</v>
       </c>
       <c r="AY80" t="n">
-        <v>199600</v>
+        <v>199300</v>
       </c>
       <c r="AZ80" t="n">
-        <v>101300</v>
+        <v>98800</v>
       </c>
       <c r="BA80" t="n">
-        <v>132100</v>
+        <v>144900</v>
       </c>
       <c r="BB80" t="n">
-        <v>191600</v>
+        <v>188600</v>
       </c>
       <c r="BC80" t="n">
-        <v>144300</v>
+        <v>149200</v>
       </c>
       <c r="BD80" t="n">
-        <v>375000</v>
+        <v>393000</v>
       </c>
       <c r="BE80" t="n">
-        <v>54200</v>
+        <v>52400</v>
       </c>
       <c r="BF80" t="n">
-        <v>71700</v>
+        <v>65500</v>
       </c>
       <c r="BG80" t="n">
-        <v>151800</v>
+        <v>147600</v>
       </c>
       <c r="BH80" t="n">
-        <v>239000</v>
+        <v>229000</v>
       </c>
       <c r="BI80" t="n">
-        <v>452000</v>
+        <v>393000</v>
       </c>
       <c r="BJ80" t="n">
-        <v>107200</v>
+        <v>99000</v>
       </c>
       <c r="BK80" t="n">
-        <v>31600</v>
+        <v>31000</v>
       </c>
       <c r="BL80" t="n">
-        <v>238000</v>
+        <v>240500</v>
       </c>
       <c r="BM80" t="n">
-        <v>22900</v>
+        <v>23000</v>
       </c>
       <c r="BN80" t="n">
-        <v>329000</v>
+        <v>288000</v>
       </c>
       <c r="BO80" t="n">
-        <v>155800</v>
+        <v>163000</v>
       </c>
       <c r="BP80" t="n">
-        <v>112000</v>
+        <v>107700</v>
       </c>
       <c r="BQ80" t="n">
-        <v>26750</v>
+        <v>26500</v>
       </c>
       <c r="BR80" t="n">
-        <v>384500</v>
+        <v>396000</v>
       </c>
       <c r="BS80" t="n">
-        <v>220500</v>
+        <v>208500</v>
       </c>
       <c r="BT80" t="n">
-        <v>134700</v>
+        <v>113500</v>
       </c>
       <c r="BU80" t="n">
-        <v>71500</v>
+        <v>73600</v>
       </c>
       <c r="BV80" t="n">
-        <v>197200</v>
+        <v>201000</v>
       </c>
       <c r="BW80" t="n">
-        <v>336000</v>
+        <v>322000</v>
       </c>
       <c r="BX80" t="n">
-        <v>49500</v>
+        <v>50900</v>
       </c>
       <c r="BY80" t="n">
-        <v>44100</v>
+        <v>40850</v>
       </c>
       <c r="BZ80" t="n">
-        <v>1139000</v>
+        <v>1069000</v>
       </c>
       <c r="CA80" t="n">
-        <v>103800</v>
+        <v>92000</v>
       </c>
       <c r="CB80" t="n">
-        <v>80200</v>
+        <v>82800</v>
       </c>
       <c r="CC80" t="n">
-        <v>123100</v>
+        <v>124400</v>
       </c>
       <c r="CD80" t="n">
-        <v>17450</v>
+        <v>15150</v>
       </c>
       <c r="CE80" t="n">
-        <v>204000</v>
+        <v>198000</v>
       </c>
       <c r="CF80" t="n">
-        <v>71100</v>
+        <v>65000</v>
       </c>
       <c r="CG80" t="n">
-        <v>93600</v>
+        <v>93200</v>
       </c>
       <c r="CH80" t="n">
-        <v>82400</v>
+        <v>79400</v>
       </c>
       <c r="CI80" t="n">
-        <v>89900</v>
+        <v>96700</v>
       </c>
       <c r="CJ80" t="n">
-        <v>14960</v>
+        <v>14620</v>
       </c>
       <c r="CK80" t="n">
         <v>130300</v>
       </c>
       <c r="CL80" t="n">
-        <v>62900</v>
+        <v>64300</v>
       </c>
       <c r="CM80" t="n">
-        <v>120900</v>
+        <v>138000</v>
       </c>
       <c r="CN80" t="n">
-        <v>629000</v>
+        <v>589000</v>
       </c>
       <c r="CO80" t="n">
-        <v>30250</v>
+        <v>27700</v>
       </c>
       <c r="CP80" t="n">
-        <v>189100</v>
+        <v>170000</v>
       </c>
       <c r="CQ80" t="n">
-        <v>48400</v>
+        <v>47050</v>
       </c>
       <c r="CR80" t="n">
-        <v>17850</v>
+        <v>18330</v>
       </c>
       <c r="CS80" t="n">
-        <v>11010</v>
+        <v>10410</v>
       </c>
       <c r="CT80" t="n">
-        <v>31900</v>
+        <v>27600</v>
       </c>
       <c r="CU80" t="n">
-        <v>68500</v>
+        <v>70800</v>
       </c>
       <c r="CV80" t="n">
-        <v>137100</v>
+        <v>128400</v>
       </c>
       <c r="CW80" t="n">
-        <v>248500</v>
+        <v>223000</v>
       </c>
       <c r="CX80" t="n">
-        <v>121900</v>
+        <v>109600</v>
       </c>
       <c r="CY80" t="n">
-        <v>38850</v>
+        <v>40900</v>
       </c>
       <c r="CZ80" t="n">
-        <v>389000</v>
+        <v>386000</v>
       </c>
       <c r="DA80" t="n">
-        <v>26050</v>
+        <v>27400</v>
       </c>
       <c r="DB80" t="n">
-        <v>10230</v>
+        <v>10190</v>
       </c>
       <c r="DC80" t="n">
-        <v>74500</v>
+        <v>67000</v>
       </c>
       <c r="DD80" t="n">
-        <v>204500</v>
+        <v>194600</v>
       </c>
       <c r="DE80" t="n">
-        <v>94600</v>
+        <v>85200</v>
       </c>
       <c r="DF80" t="n">
-        <v>155300</v>
+        <v>140800</v>
       </c>
       <c r="DG80" t="n">
-        <v>254500</v>
+        <v>196700</v>
       </c>
       <c r="DH80" t="n">
-        <v>142200</v>
+        <v>135700</v>
       </c>
       <c r="DI80" t="n">
-        <v>100500</v>
+        <v>92000</v>
       </c>
       <c r="DJ80" t="n">
-        <v>4650</v>
+        <v>4540</v>
       </c>
       <c r="DK80" t="n">
-        <v>102200</v>
+        <v>92700</v>
       </c>
       <c r="DL80" t="n">
-        <v>453500</v>
+        <v>420000</v>
       </c>
       <c r="DM80" t="n">
-        <v>46600</v>
+        <v>46900</v>
       </c>
       <c r="DN80" t="n">
-        <v>87000</v>
+        <v>86900</v>
       </c>
       <c r="DO80" t="n">
-        <v>3605</v>
+        <v>3490</v>
       </c>
       <c r="DP80" t="n">
-        <v>197800</v>
+        <v>194300</v>
       </c>
       <c r="DQ80" t="n">
-        <v>245000</v>
+        <v>246500</v>
       </c>
       <c r="DR80" t="n">
-        <v>167100</v>
+        <v>157400</v>
       </c>
       <c r="DS80" t="n">
-        <v>26900</v>
+        <v>26550</v>
       </c>
       <c r="DT80" t="n">
         <v>120000</v>
       </c>
       <c r="DU80" t="n">
-        <v>38150</v>
+        <v>38300</v>
       </c>
       <c r="DV80" t="n">
-        <v>66200</v>
+        <v>59500</v>
       </c>
       <c r="DW80" t="n">
-        <v>14610</v>
+        <v>14410</v>
       </c>
       <c r="DX80" t="n">
-        <v>47050</v>
+        <v>44550</v>
       </c>
       <c r="DY80" t="n">
-        <v>37550</v>
+        <v>36300</v>
       </c>
       <c r="DZ80" t="n">
-        <v>20200</v>
+        <v>18630</v>
       </c>
       <c r="EA80" t="n">
-        <v>33050</v>
+        <v>32400</v>
       </c>
       <c r="EB80" t="n">
+        <v>43100</v>
+      </c>
+      <c r="EC80" t="n">
+        <v>52800</v>
+      </c>
+      <c r="ED80" t="n">
+        <v>79000</v>
+      </c>
+      <c r="EE80" t="n">
+        <v>123500</v>
+      </c>
+      <c r="EF80" t="n">
+        <v>35450</v>
+      </c>
+      <c r="EG80" t="n">
+        <v>184800</v>
+      </c>
+      <c r="EH80" t="n">
+        <v>18410</v>
+      </c>
+      <c r="EI80" t="n">
+        <v>5160</v>
+      </c>
+      <c r="EJ80" t="n">
+        <v>72100</v>
+      </c>
+      <c r="EK80" t="n">
+        <v>244500</v>
+      </c>
+      <c r="EL80" t="n">
+        <v>27300</v>
+      </c>
+      <c r="EM80" t="n">
+        <v>68900</v>
+      </c>
+      <c r="EN80" t="n">
+        <v>36500</v>
+      </c>
+      <c r="EO80" t="n">
+        <v>61000</v>
+      </c>
+      <c r="EP80" t="n">
+        <v>143100</v>
+      </c>
+      <c r="EQ80" t="n">
+        <v>54400</v>
+      </c>
+      <c r="ER80" t="n">
+        <v>25500</v>
+      </c>
+      <c r="ES80" t="n">
+        <v>149400</v>
+      </c>
+      <c r="ET80" t="n">
+        <v>107600</v>
+      </c>
+      <c r="EU80" t="n">
+        <v>16760</v>
+      </c>
+      <c r="EV80" t="n">
+        <v>208500</v>
+      </c>
+      <c r="EW80" t="n">
+        <v>191200</v>
+      </c>
+      <c r="EX80" t="n">
+        <v>60200</v>
+      </c>
+      <c r="EY80" t="n">
+        <v>13660</v>
+      </c>
+      <c r="EZ80" t="n">
+        <v>25250</v>
+      </c>
+      <c r="FA80" t="n">
+        <v>46950</v>
+      </c>
+      <c r="FB80" t="n">
+        <v>22800</v>
+      </c>
+      <c r="FC80" t="n">
+        <v>44800</v>
+      </c>
+      <c r="FD80" t="n">
+        <v>45800</v>
+      </c>
+      <c r="FE80" t="n">
+        <v>32700</v>
+      </c>
+      <c r="FF80" t="n">
+        <v>79700</v>
+      </c>
+      <c r="FG80" t="n">
+        <v>5850</v>
+      </c>
+      <c r="FH80" t="n">
+        <v>6390</v>
+      </c>
+      <c r="FI80" t="n">
+        <v>13950</v>
+      </c>
+      <c r="FJ80" t="n">
+        <v>26400</v>
+      </c>
+      <c r="FK80" t="n">
+        <v>349500</v>
+      </c>
+      <c r="FL80" t="n">
+        <v>18610</v>
+      </c>
+      <c r="FM80" t="n">
+        <v>126400</v>
+      </c>
+      <c r="FN80" t="n">
+        <v>40800</v>
+      </c>
+      <c r="FO80" t="n">
+        <v>57600</v>
+      </c>
+      <c r="FP80" t="n">
         <v>43550</v>
       </c>
-      <c r="EC80" t="n">
-        <v>57400</v>
-      </c>
-      <c r="ED80" t="n">
-        <v>77600</v>
-      </c>
-      <c r="EE80" t="n">
-        <v>117400</v>
-      </c>
-      <c r="EF80" t="n">
-        <v>36650</v>
-      </c>
-      <c r="EG80" t="n">
-        <v>191000</v>
-      </c>
-      <c r="EH80" t="n">
-        <v>17850</v>
-      </c>
-      <c r="EI80" t="n">
-        <v>5250</v>
-      </c>
-      <c r="EJ80" t="n">
-        <v>73000</v>
-      </c>
-      <c r="EK80" t="n">
-        <v>248500</v>
-      </c>
-      <c r="EL80" t="n">
-        <v>31850</v>
-      </c>
-      <c r="EM80" t="n">
-        <v>69500</v>
-      </c>
-      <c r="EN80" t="n">
-        <v>38100</v>
-      </c>
-      <c r="EO80" t="n">
-        <v>61800</v>
-      </c>
-      <c r="EP80" t="n">
-        <v>155500</v>
-      </c>
-      <c r="EQ80" t="n">
-        <v>55700</v>
-      </c>
-      <c r="ER80" t="n">
-        <v>25900</v>
-      </c>
-      <c r="ES80" t="n">
-        <v>156900</v>
-      </c>
-      <c r="ET80" t="n">
-        <v>106500</v>
-      </c>
-      <c r="EU80" t="n">
-        <v>18320</v>
-      </c>
-      <c r="EV80" t="n">
-        <v>197900</v>
-      </c>
-      <c r="EW80" t="n">
-        <v>189300</v>
-      </c>
-      <c r="EX80" t="n">
-        <v>63300</v>
-      </c>
-      <c r="EY80" t="n">
-        <v>13850</v>
-      </c>
-      <c r="EZ80" t="n">
-        <v>25050</v>
-      </c>
-      <c r="FA80" t="n">
-        <v>44650</v>
-      </c>
-      <c r="FB80" t="n">
-        <v>23400</v>
-      </c>
-      <c r="FC80" t="n">
-        <v>49550</v>
-      </c>
-      <c r="FD80" t="n">
-        <v>45300</v>
-      </c>
-      <c r="FE80" t="n">
-        <v>33400</v>
-      </c>
-      <c r="FF80" t="n">
-        <v>81800</v>
-      </c>
-      <c r="FG80" t="n">
-        <v>7800</v>
-      </c>
-      <c r="FH80" t="n">
-        <v>5520</v>
-      </c>
-      <c r="FI80" t="n">
-        <v>14000</v>
-      </c>
-      <c r="FJ80" t="n">
-        <v>25950</v>
-      </c>
-      <c r="FK80" t="n">
-        <v>356000</v>
-      </c>
-      <c r="FL80" t="n">
-        <v>18810</v>
-      </c>
-      <c r="FM80" t="n">
-        <v>123600</v>
-      </c>
-      <c r="FN80" t="n">
-        <v>35850</v>
-      </c>
-      <c r="FO80" t="n">
-        <v>61600</v>
-      </c>
-      <c r="FP80" t="n">
-        <v>45950</v>
-      </c>
       <c r="FQ80" t="n">
-        <v>35150</v>
+        <v>32450</v>
       </c>
       <c r="FR80" t="n">
-        <v>216500</v>
+        <v>222000</v>
       </c>
       <c r="FS80" t="n">
-        <v>50400</v>
+        <v>47800</v>
       </c>
       <c r="FT80" t="n">
-        <v>172700</v>
+        <v>181100</v>
       </c>
       <c r="FU80" t="n">
-        <v>97400</v>
+        <v>100800</v>
       </c>
       <c r="FV80" t="n">
-        <v>63100</v>
+        <v>58500</v>
       </c>
       <c r="FW80" t="n">
-        <v>35600</v>
+        <v>32250</v>
       </c>
       <c r="FX80" t="n">
-        <v>24300</v>
+        <v>25000</v>
       </c>
       <c r="FY80" t="n">
-        <v>464000</v>
+        <v>415500</v>
       </c>
       <c r="FZ80" t="n">
-        <v>48250</v>
+        <v>45750</v>
       </c>
       <c r="GA80" t="n">
-        <v>65100</v>
+        <v>62100</v>
       </c>
       <c r="GB80" t="n">
-        <v>13240</v>
+        <v>12650</v>
       </c>
       <c r="GC80" t="n">
-        <v>73800</v>
+        <v>70300</v>
       </c>
       <c r="GD80" t="n">
-        <v>8580</v>
+        <v>7990</v>
       </c>
       <c r="GE80" t="n">
-        <v>5710</v>
+        <v>5650</v>
       </c>
       <c r="GF80" t="n">
-        <v>73900</v>
+        <v>72500</v>
       </c>
       <c r="GG80" t="n">
-        <v>61900</v>
+        <v>57600</v>
       </c>
       <c r="GH80" t="n">
         <v>39850</v>
       </c>
       <c r="GI80" t="n">
-        <v>55900</v>
+        <v>53600</v>
       </c>
       <c r="GJ80" t="n">
-        <v>565000</v>
+        <v>467500</v>
       </c>
       <c r="GK80" t="n">
+        <v>26050</v>
+      </c>
+      <c r="GL80" t="n">
+        <v>35650</v>
+      </c>
+      <c r="GM80" t="n">
+        <v>15560</v>
+      </c>
+      <c r="GN80" t="n">
+        <v>121900</v>
+      </c>
+      <c r="GO80" t="n">
+        <v>33350</v>
+      </c>
+      <c r="GP80" t="n">
+        <v>7080</v>
+      </c>
+      <c r="GQ80" t="n">
+        <v>11690</v>
+      </c>
+      <c r="GR80" t="n">
+        <v>52000</v>
+      </c>
+      <c r="GS80" t="n">
+        <v>122800</v>
+      </c>
+      <c r="GT80" t="n">
+        <v>276500</v>
+      </c>
+      <c r="GU80" t="n">
+        <v>112400</v>
+      </c>
+      <c r="GV80" t="n">
+        <v>80000</v>
+      </c>
+      <c r="GW80" t="n">
+        <v>187900</v>
+      </c>
+      <c r="GX80" t="n">
+        <v>397000</v>
+      </c>
+      <c r="GY80" t="n">
+        <v>62100</v>
+      </c>
+      <c r="GZ80" t="n">
+        <v>140700</v>
+      </c>
+      <c r="HA80" t="n">
+        <v>72300</v>
+      </c>
+      <c r="HB80" t="n">
+        <v>195400</v>
+      </c>
+      <c r="HC80" t="n">
+        <v>35300</v>
+      </c>
+      <c r="HD80" t="n">
+        <v>184100</v>
+      </c>
+      <c r="HE80" t="n">
+        <v>344000</v>
+      </c>
+      <c r="HF80" t="n">
+        <v>107400</v>
+      </c>
+      <c r="HG80" t="n">
+        <v>75600</v>
+      </c>
+      <c r="HH80" t="n">
+        <v>103700</v>
+      </c>
+      <c r="HI80" t="n">
+        <v>68700</v>
+      </c>
+      <c r="HJ80" t="n">
+        <v>70400</v>
+      </c>
+      <c r="HK80" t="n">
+        <v>146800</v>
+      </c>
+      <c r="HL80" t="n">
+        <v>42500</v>
+      </c>
+      <c r="HM80" t="n">
+        <v>194300</v>
+      </c>
+      <c r="HN80" t="n">
+        <v>336500</v>
+      </c>
+      <c r="HO80" t="n">
+        <v>61700</v>
+      </c>
+      <c r="HP80" t="n">
+        <v>145000</v>
+      </c>
+      <c r="HQ80" t="n">
+        <v>199900</v>
+      </c>
+      <c r="HR80" t="n">
+        <v>44100</v>
+      </c>
+      <c r="HS80" t="n">
+        <v>81900</v>
+      </c>
+      <c r="HT80" t="n">
+        <v>145600</v>
+      </c>
+      <c r="HU80" t="n">
+        <v>39300</v>
+      </c>
+      <c r="HV80" t="n">
+        <v>282500</v>
+      </c>
+      <c r="HW80" t="n">
+        <v>239500</v>
+      </c>
+      <c r="HX80" t="n">
+        <v>143400</v>
+      </c>
+      <c r="HY80" t="n">
+        <v>35750</v>
+      </c>
+      <c r="HZ80" t="n">
+        <v>119200</v>
+      </c>
+      <c r="IA80" t="n">
+        <v>215000</v>
+      </c>
+      <c r="IB80" t="n">
+        <v>19220</v>
+      </c>
+      <c r="IC80" t="n">
+        <v>124300</v>
+      </c>
+      <c r="ID80" t="n">
+        <v>108300</v>
+      </c>
+      <c r="IE80" t="n">
+        <v>136600</v>
+      </c>
+      <c r="IF80" t="n">
+        <v>36050</v>
+      </c>
+      <c r="IG80" t="n">
+        <v>291500</v>
+      </c>
+      <c r="IH80" t="n">
+        <v>43600</v>
+      </c>
+      <c r="II80" t="n">
+        <v>34150</v>
+      </c>
+      <c r="IJ80" t="n">
+        <v>162800</v>
+      </c>
+      <c r="IK80" t="n">
+        <v>26400</v>
+      </c>
+      <c r="IL80" t="n">
+        <v>71000</v>
+      </c>
+      <c r="IM80" t="n">
+        <v>10300</v>
+      </c>
+      <c r="IN80" t="n">
+        <v>86900</v>
+      </c>
+      <c r="IO80" t="n">
+        <v>9850</v>
+      </c>
+      <c r="IP80" t="n">
+        <v>258000</v>
+      </c>
+      <c r="IQ80" t="n">
+        <v>39800</v>
+      </c>
+      <c r="IR80" t="n">
+        <v>46650</v>
+      </c>
+      <c r="IS80" t="n">
+        <v>69100</v>
+      </c>
+      <c r="IT80" t="n">
+        <v>52900</v>
+      </c>
+      <c r="IU80" t="n">
+        <v>71900</v>
+      </c>
+      <c r="IV80" t="n">
+        <v>66000</v>
+      </c>
+      <c r="IW80" t="n">
+        <v>49200</v>
+      </c>
+      <c r="IX80" t="n">
+        <v>25000</v>
+      </c>
+      <c r="IY80" t="n">
+        <v>17830</v>
+      </c>
+      <c r="IZ80" t="n">
+        <v>21150</v>
+      </c>
+      <c r="JA80" t="n">
         <v>26800</v>
       </c>
-      <c r="GL80" t="n">
-        <v>37100</v>
-      </c>
-      <c r="GM80" t="n">
-        <v>17730</v>
-      </c>
-      <c r="GN80" t="n">
-        <v>131900</v>
-      </c>
-      <c r="GO80" t="n">
-        <v>34550</v>
-      </c>
-      <c r="GP80" t="n">
-        <v>7160</v>
-      </c>
-      <c r="GQ80" t="n">
-        <v>13740</v>
-      </c>
-      <c r="GR80" t="n">
-        <v>42850</v>
-      </c>
-      <c r="GS80" t="n">
-        <v>123200</v>
-      </c>
-      <c r="GT80" t="n">
-        <v>324000</v>
-      </c>
-      <c r="GU80" t="n">
-        <v>121600</v>
-      </c>
-      <c r="GV80" t="n">
-        <v>85800</v>
-      </c>
-      <c r="GW80" t="n">
-        <v>191900</v>
-      </c>
-      <c r="GX80" t="n">
-        <v>453500</v>
-      </c>
-      <c r="GY80" t="n">
-        <v>90000</v>
-      </c>
-      <c r="GZ80" t="n">
-        <v>125000</v>
-      </c>
-      <c r="HA80" t="n">
-        <v>73800</v>
-      </c>
-      <c r="HB80" t="n">
-        <v>189400</v>
-      </c>
-      <c r="HC80" t="n">
-        <v>36600</v>
-      </c>
-      <c r="HD80" t="n">
-        <v>199600</v>
-      </c>
-      <c r="HE80" t="n">
-        <v>378500</v>
-      </c>
-      <c r="HF80" t="n">
-        <v>122700</v>
-      </c>
-      <c r="HG80" t="n">
-        <v>81800</v>
-      </c>
-      <c r="HH80" t="n">
-        <v>120300</v>
-      </c>
-      <c r="HI80" t="n">
-        <v>84300</v>
-      </c>
-      <c r="HJ80" t="n">
-        <v>76800</v>
-      </c>
-      <c r="HK80" t="n">
-        <v>165700</v>
-      </c>
-      <c r="HL80" t="n">
-        <v>44400</v>
-      </c>
-      <c r="HM80" t="n">
-        <v>177700</v>
-      </c>
-      <c r="HN80" t="n">
-        <v>319500</v>
-      </c>
-      <c r="HO80" t="n">
-        <v>61100</v>
-      </c>
-      <c r="HP80" t="n">
-        <v>151200</v>
-      </c>
-      <c r="HQ80" t="n">
-        <v>218000</v>
-      </c>
-      <c r="HR80" t="n">
-        <v>48500</v>
-      </c>
-      <c r="HS80" t="n">
-        <v>89100</v>
-      </c>
-      <c r="HT80" t="n">
-        <v>166200</v>
-      </c>
-      <c r="HU80" t="n">
-        <v>47350</v>
-      </c>
-      <c r="HV80" t="n">
-        <v>269500</v>
-      </c>
-      <c r="HW80" t="n">
-        <v>240500</v>
-      </c>
-      <c r="HX80" t="n">
-        <v>136200</v>
-      </c>
-      <c r="HY80" t="n">
-        <v>39750</v>
-      </c>
-      <c r="HZ80" t="n">
-        <v>111600</v>
-      </c>
-      <c r="IA80" t="n">
-        <v>232000</v>
-      </c>
-      <c r="IB80" t="n">
-        <v>23250</v>
-      </c>
-      <c r="IC80" t="n">
-        <v>123600</v>
-      </c>
-      <c r="ID80" t="n">
-        <v>103400</v>
-      </c>
-      <c r="IE80" t="n">
-        <v>123200</v>
-      </c>
-      <c r="IF80" t="n">
-        <v>37600</v>
-      </c>
-      <c r="IG80" t="n">
-        <v>311500</v>
-      </c>
-      <c r="IH80" t="n">
-        <v>47150</v>
-      </c>
-      <c r="II80" t="n">
-        <v>37050</v>
-      </c>
-      <c r="IJ80" t="n">
-        <v>164500</v>
-      </c>
-      <c r="IK80" t="n">
-        <v>28800</v>
-      </c>
-      <c r="IL80" t="n">
-        <v>72700</v>
-      </c>
-      <c r="IM80" t="n">
-        <v>12600</v>
-      </c>
-      <c r="IN80" t="n">
-        <v>99900</v>
-      </c>
-      <c r="IO80" t="n">
-        <v>11210</v>
-      </c>
-      <c r="IP80" t="n">
-        <v>269500</v>
-      </c>
-      <c r="IQ80" t="n">
-        <v>41000</v>
-      </c>
-      <c r="IR80" t="n">
-        <v>50700</v>
-      </c>
-      <c r="IS80" t="n">
-        <v>77500</v>
-      </c>
-      <c r="IT80" t="n">
-        <v>56600</v>
-      </c>
-      <c r="IU80" t="n">
-        <v>83300</v>
-      </c>
-      <c r="IV80" t="n">
-        <v>74000</v>
-      </c>
-      <c r="IW80" t="n">
-        <v>43900</v>
-      </c>
-      <c r="IX80" t="n">
+      <c r="JB80" t="n">
+        <v>28550</v>
+      </c>
+      <c r="JC80" t="n">
+        <v>42650</v>
+      </c>
+      <c r="JD80" t="n">
+        <v>16790</v>
+      </c>
+      <c r="JE80" t="n">
+        <v>28900</v>
+      </c>
+      <c r="JF80" t="n">
+        <v>46250</v>
+      </c>
+      <c r="JG80" t="n">
+        <v>30050</v>
+      </c>
+      <c r="JH80" t="n">
+        <v>34750</v>
+      </c>
+      <c r="JI80" t="n">
+        <v>76300</v>
+      </c>
+      <c r="JJ80" t="n">
+        <v>36950</v>
+      </c>
+      <c r="JK80" t="n">
+        <v>30150</v>
+      </c>
+      <c r="JL80" t="n">
+        <v>10570</v>
+      </c>
+      <c r="JM80" t="n">
+        <v>9760</v>
+      </c>
+      <c r="JN80" t="n">
+        <v>38800</v>
+      </c>
+      <c r="JO80" t="n">
+        <v>18890</v>
+      </c>
+      <c r="JP80" t="n">
+        <v>54600</v>
+      </c>
+      <c r="JQ80" t="n">
+        <v>29000</v>
+      </c>
+      <c r="JR80" t="n">
+        <v>45400</v>
+      </c>
+      <c r="JS80" t="n">
+        <v>37850</v>
+      </c>
+      <c r="JT80" t="n">
+        <v>15500</v>
+      </c>
+      <c r="JU80" t="n">
+        <v>43800</v>
+      </c>
+      <c r="JV80" t="n">
+        <v>77900</v>
+      </c>
+      <c r="JW80" t="n">
+        <v>9120</v>
+      </c>
+      <c r="JX80" t="n">
+        <v>44850</v>
+      </c>
+      <c r="JY80" t="n">
+        <v>7850</v>
+      </c>
+      <c r="JZ80" t="n">
+        <v>7590</v>
+      </c>
+      <c r="KA80" t="n">
+        <v>84800</v>
+      </c>
+      <c r="KB80" t="n">
+        <v>14110</v>
+      </c>
+      <c r="KC80" t="n">
+        <v>9980</v>
+      </c>
+      <c r="KD80" t="n">
+        <v>5620</v>
+      </c>
+      <c r="KE80" t="n">
+        <v>6390</v>
+      </c>
+      <c r="KF80" t="n">
+        <v>19290</v>
+      </c>
+      <c r="KG80" t="n">
+        <v>11510</v>
+      </c>
+      <c r="KH80" t="n">
+        <v>11900</v>
+      </c>
+      <c r="KI80" t="n">
+        <v>23100</v>
+      </c>
+      <c r="KJ80" t="n">
+        <v>86300</v>
+      </c>
+      <c r="KK80" t="n">
+        <v>29000</v>
+      </c>
+      <c r="KL80" t="n">
+        <v>20700</v>
+      </c>
+      <c r="KM80" t="n">
+        <v>61200</v>
+      </c>
+      <c r="KN80" t="n">
+        <v>27350</v>
+      </c>
+      <c r="KO80" t="n">
+        <v>10040</v>
+      </c>
+      <c r="KP80" t="n">
+        <v>40200</v>
+      </c>
+      <c r="KQ80" t="n">
+        <v>62900</v>
+      </c>
+      <c r="KR80" t="n">
+        <v>29900</v>
+      </c>
+      <c r="KS80" t="n">
+        <v>31750</v>
+      </c>
+      <c r="KT80" t="n">
+        <v>15080</v>
+      </c>
+      <c r="KU80" t="n">
+        <v>38300</v>
+      </c>
+      <c r="KV80" t="n">
+        <v>18360</v>
+      </c>
+      <c r="KW80" t="n">
+        <v>41150</v>
+      </c>
+      <c r="KX80" t="n">
+        <v>32100</v>
+      </c>
+      <c r="KY80" t="n">
+        <v>27700</v>
+      </c>
+      <c r="KZ80" t="n">
+        <v>18290</v>
+      </c>
+      <c r="LA80" t="n">
+        <v>42800</v>
+      </c>
+      <c r="LB80" t="n">
+        <v>54200</v>
+      </c>
+      <c r="LC80" t="n">
+        <v>29300</v>
+      </c>
+      <c r="LD80" t="n">
+        <v>14570</v>
+      </c>
+      <c r="LE80" t="n">
+        <v>25900</v>
+      </c>
+      <c r="LF80" t="n">
+        <v>6520</v>
+      </c>
+      <c r="LG80" t="n">
+        <v>61200</v>
+      </c>
+      <c r="LH80" t="n">
+        <v>17850</v>
+      </c>
+      <c r="LI80" t="n">
+        <v>9900</v>
+      </c>
+      <c r="LJ80" t="n">
+        <v>23400</v>
+      </c>
+      <c r="LK80" t="n">
+        <v>28750</v>
+      </c>
+      <c r="LL80" t="n">
+        <v>49750</v>
+      </c>
+      <c r="LM80" t="n">
+        <v>20400</v>
+      </c>
+      <c r="LN80" t="n">
+        <v>30750</v>
+      </c>
+      <c r="LO80" t="n">
+        <v>41150</v>
+      </c>
+      <c r="LP80" t="n">
+        <v>9440</v>
+      </c>
+      <c r="LQ80" t="n">
+        <v>133400</v>
+      </c>
+      <c r="LR80" t="n">
+        <v>16640</v>
+      </c>
+      <c r="LS80" t="n">
         <v>25200</v>
       </c>
-      <c r="IY80" t="n">
-        <v>22150</v>
-      </c>
-      <c r="IZ80" t="n">
-        <v>23950</v>
-      </c>
-      <c r="JA80" t="n">
-        <v>29000</v>
-      </c>
-      <c r="JB80" t="n">
-        <v>29000</v>
-      </c>
-      <c r="JC80" t="n">
+      <c r="LT80" t="n">
+        <v>7260</v>
+      </c>
+      <c r="LU80" t="n">
+        <v>52400</v>
+      </c>
+      <c r="LV80" t="n">
+        <v>22550</v>
+      </c>
+      <c r="LW80" t="n">
+        <v>40250</v>
+      </c>
+      <c r="LX80" t="n">
+        <v>66600</v>
+      </c>
+      <c r="LY80" t="n">
+        <v>8380</v>
+      </c>
+      <c r="LZ80" t="n">
+        <v>35050</v>
+      </c>
+      <c r="MA80" t="n">
+        <v>26550</v>
+      </c>
+      <c r="MB80" t="n">
+        <v>25800</v>
+      </c>
+      <c r="MC80" t="n">
+        <v>9090</v>
+      </c>
+      <c r="MD80" t="n">
         <v>48350</v>
       </c>
-      <c r="JD80" t="n">
-        <v>18790</v>
-      </c>
-      <c r="JE80" t="n">
-        <v>31100</v>
-      </c>
-      <c r="JF80" t="n">
-        <v>52100</v>
-      </c>
-      <c r="JG80" t="n">
-        <v>36000</v>
-      </c>
-      <c r="JH80" t="n">
-        <v>38950</v>
-      </c>
-      <c r="JI80" t="n">
-        <v>81600</v>
-      </c>
-      <c r="JJ80" t="n">
+      <c r="ME80" t="n">
         <v>38900</v>
       </c>
-      <c r="JK80" t="n">
-        <v>31050</v>
-      </c>
-      <c r="JL80" t="n">
-        <v>11840</v>
-      </c>
-      <c r="JM80" t="n">
-        <v>10360</v>
-      </c>
-      <c r="JN80" t="n">
-        <v>40800</v>
-      </c>
-      <c r="JO80" t="n">
-        <v>21800</v>
-      </c>
-      <c r="JP80" t="n">
-        <v>56400</v>
-      </c>
-      <c r="JQ80" t="n">
-        <v>34100</v>
-      </c>
-      <c r="JR80" t="n">
-        <v>48700</v>
-      </c>
-      <c r="JS80" t="n">
-        <v>42250</v>
-      </c>
-      <c r="JT80" t="n">
-        <v>17810</v>
-      </c>
-      <c r="JU80" t="n">
-        <v>47750</v>
-      </c>
-      <c r="JV80" t="n">
-        <v>88100</v>
-      </c>
-      <c r="JW80" t="n">
-        <v>10200</v>
-      </c>
-      <c r="JX80" t="n">
-        <v>48550</v>
-      </c>
-      <c r="JY80" t="n">
-        <v>8340</v>
-      </c>
-      <c r="JZ80" t="n">
-        <v>8260</v>
-      </c>
-      <c r="KA80" t="n">
-        <v>83000</v>
-      </c>
-      <c r="KB80" t="n">
-        <v>16650</v>
-      </c>
-      <c r="KC80" t="n">
-        <v>10780</v>
-      </c>
-      <c r="KD80" t="n">
-        <v>5350</v>
-      </c>
-      <c r="KE80" t="n">
-        <v>7320</v>
-      </c>
-      <c r="KF80" t="n">
-        <v>19180</v>
-      </c>
-      <c r="KG80" t="n">
-        <v>12670</v>
-      </c>
-      <c r="KH80" t="n">
-        <v>12820</v>
-      </c>
-      <c r="KI80" t="n">
-        <v>22500</v>
-      </c>
-      <c r="KJ80" t="n">
-        <v>85000</v>
-      </c>
-      <c r="KK80" t="n">
-        <v>31150</v>
-      </c>
-      <c r="KL80" t="n">
-        <v>22750</v>
-      </c>
-      <c r="KM80" t="n">
-        <v>69000</v>
-      </c>
-      <c r="KN80" t="n">
-        <v>29500</v>
-      </c>
-      <c r="KO80" t="n">
-        <v>10840</v>
-      </c>
-      <c r="KP80" t="n">
-        <v>42200</v>
-      </c>
-      <c r="KQ80" t="n">
-        <v>72500</v>
-      </c>
-      <c r="KR80" t="n">
-        <v>31850</v>
-      </c>
-      <c r="KS80" t="n">
-        <v>30150</v>
-      </c>
-      <c r="KT80" t="n">
-        <v>17560</v>
-      </c>
-      <c r="KU80" t="n">
-        <v>75200</v>
-      </c>
-      <c r="KV80" t="n">
-        <v>21550</v>
-      </c>
-      <c r="KW80" t="n">
-        <v>42500</v>
-      </c>
-      <c r="KX80" t="n">
-        <v>35650</v>
-      </c>
-      <c r="KY80" t="n">
-        <v>31000</v>
-      </c>
-      <c r="KZ80" t="n">
-        <v>18970</v>
-      </c>
-      <c r="LA80" t="n">
-        <v>45200</v>
-      </c>
-      <c r="LB80" t="n">
-        <v>52500</v>
-      </c>
-      <c r="LC80" t="n">
-        <v>32200</v>
-      </c>
-      <c r="LD80" t="n">
-        <v>11700</v>
-      </c>
-      <c r="LE80" t="n">
-        <v>26500</v>
-      </c>
-      <c r="LF80" t="n">
-        <v>7260</v>
-      </c>
-      <c r="LG80" t="n">
-        <v>71700</v>
-      </c>
-      <c r="LH80" t="n">
-        <v>18500</v>
-      </c>
-      <c r="LI80" t="n">
-        <v>10790</v>
-      </c>
-      <c r="LJ80" t="n">
-        <v>26950</v>
-      </c>
-      <c r="LK80" t="n">
-        <v>31500</v>
-      </c>
-      <c r="LL80" t="n">
-        <v>57200</v>
-      </c>
-      <c r="LM80" t="n">
-        <v>22400</v>
-      </c>
-      <c r="LN80" t="n">
-        <v>31450</v>
-      </c>
-      <c r="LO80" t="n">
-        <v>44900</v>
-      </c>
-      <c r="LP80" t="n">
-        <v>10680</v>
-      </c>
-      <c r="LQ80" t="n">
-        <v>132800</v>
-      </c>
-      <c r="LR80" t="n">
-        <v>18830</v>
-      </c>
-      <c r="LS80" t="n">
-        <v>27300</v>
-      </c>
-      <c r="LT80" t="n">
-        <v>7960</v>
-      </c>
-      <c r="LU80" t="n">
+      <c r="MF80" t="n">
+        <v>14960</v>
+      </c>
+      <c r="MG80" t="n">
+        <v>41600</v>
+      </c>
+      <c r="MH80" t="n">
+        <v>43850</v>
+      </c>
+      <c r="MI80" t="n">
+        <v>47300</v>
+      </c>
+      <c r="MJ80" t="n">
+        <v>7280</v>
+      </c>
+      <c r="MK80" t="n">
         <v>55500</v>
       </c>
-      <c r="LV80" t="n">
+      <c r="ML80" t="n">
+        <v>15310</v>
+      </c>
+      <c r="MM80" t="n">
         <v>23750</v>
-      </c>
-      <c r="LW80" t="n">
-        <v>42150</v>
-      </c>
-      <c r="LX80" t="n">
-        <v>66200</v>
-      </c>
-      <c r="LY80" t="n">
-        <v>8970</v>
-      </c>
-      <c r="LZ80" t="n">
-        <v>36150</v>
-      </c>
-      <c r="MA80" t="n">
-        <v>29450</v>
-      </c>
-      <c r="MB80" t="n">
-        <v>28000</v>
-      </c>
-      <c r="MC80" t="n">
-        <v>10060</v>
-      </c>
-      <c r="MD80" t="n">
-        <v>36650</v>
-      </c>
-      <c r="ME80" t="n">
-        <v>45000</v>
-      </c>
-      <c r="MF80" t="n">
-        <v>17130</v>
-      </c>
-      <c r="MG80" t="n">
-        <v>47400</v>
-      </c>
-      <c r="MH80" t="n">
-        <v>46450</v>
-      </c>
-      <c r="MI80" t="n">
-        <v>48700</v>
-      </c>
-      <c r="MJ80" t="n">
-        <v>7500</v>
-      </c>
-      <c r="MK80" t="n">
-        <v>54800</v>
-      </c>
-      <c r="ML80" t="n">
-        <v>17920</v>
-      </c>
-      <c r="MM80" t="n">
-        <v>33300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>